<commit_message>
chore: update conference list 2026-06-01
</commit_message>
<xml_diff>
--- a/public/conference_list.xlsx
+++ b/public/conference_list.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G181"/>
+  <dimension ref="A1:G179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,64 +456,64 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026 Climate Finance &amp; Policy (CFP-2026)</t>
+          <t>EUROFIDAI-ESSEC Paris December Finance Meeting</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-12-17</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-12-17</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bari, Italy</t>
+          <t>Pullman Paris Montparnasse Hotel</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>75€</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>AI-driven Climate Risk Assessment and Prediction, Big Data and ESG Decision-making, Carbon Border Adjustment Mechanisms, Carbon Finance and Pricing, Climate Change and Corporate Behavior, Climate Finance for Energy Efficiency, Carbon Taxes, Climate Agreements and Frameworks, Climate Funds and Public Finance, Climate Risk Assessment and Disclosure, ESG Measurement, Ratings &amp; Data Quality, Financing Climate Adaptation and Resilience, Green Finance, Green Bonds and Socially Responsible Bonds, Just Transition, Nature, Biodiversity &amp; Finance, Role of Technology in Climate Finance, Sustainable Investing, Sustainability Regulation &amp; Political Economy</t>
+          <t>All areas of finance</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026 Global AI Finance Research Conference</t>
+          <t>Chicago Fed/University of Chicago Conference on Municipal Bond Markets</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-12-14</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-12-15</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Taipei, Taiwan</t>
+          <t>Federal Reserve Bank of Chicago</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -523,71 +523,71 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Artificial Intelligence (AI), Big Data and Machine Learning, Blockchain and Cryptocurrencies, Security Token Offerings (STOs) and Initial Coin Offerings (ICOs), Decentralized Finance (DeFi), Peer-to-peer lending, FinTech regulation, High-frequency trading and market liquidity, Green FinTech</t>
+          <t>Unpublished and policy-relevant research papers on municipal bond markets, primary market frictions, secondary market frictions, role of retail investors, government policies affecting bond price formation, effects of state and federal policies on government access to external finance</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>37th Annual Conference of the Academy of Behavioral Finance &amp; Economics</t>
+          <t>SFS Cavalcade Asia-Pacific 2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-12-09</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Santa Monica, California, USA</t>
+          <t>City University of Hong Kong</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>$99.00 USD</t>
+          <t>$75 USD</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Behavioral/Cognitive Finance &amp; Economics, Neuroscience/Neuromorphic Computing, Political Economy, Biological Anthropology, Brain-Computer Interfaces</t>
+          <t>Financial studies, Asset pricing, Corporate finance</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Colorado Finance Summit 2026</t>
+          <t>2026 CLIMATE FINANCE &amp; POLICY (CFP-2026)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-12-10</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-12-13</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Vail, Colorado</t>
+          <t>Bari, Italy</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -597,182 +597,182 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>All areas of finance, theoretical and empirical contributions</t>
+          <t>AI-driven Climate Risk Assessment and Prediction, Big Data and ESG Decision-making, Carbon Border Adjustment Mechanisms, Carbon Finance and Pricing, Climate Change and Corporate Behavior, Climate Finance for Energy Efficiency, Carbon Taxes, Climate Agreements and Frameworks, Climate Funds and Public Finance, Climate Risk Assessment and Disclosure, ESG Measurement, Ratings &amp; Data Quality, Financing Climate Adaptation and Resilience, Green Finance, Green Bonds and Socially Responsible Bonds, Just Transition, Nature, Biodiversity &amp; Finance, Role of Technology in Climate Finance, Sustainable Investing, Sustainability Regulation &amp; Political Economy</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026 UNSW Asset Pricing Workshop</t>
+          <t>2026 Global AI Finance Research Conference</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-12-14</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-12-04</t>
+          <t>2026-12-15</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Sydney (NSW, Australia)</t>
+          <t>Taipei, Taiwan</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0 AUD</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>All areas of Finance, with a special focus on Asset Pricing</t>
+          <t>Artificial Intelligence (AI), Big Data and Machine Learning, Blockchain and Cryptocurrencies, Security Token Offerings (STOs) and Initial Coin Offerings (ICOs), Decentralized Finance (DeFi), Peer-to-peer lending, FinTech regulation, High-frequency trading and market liquidity, Green FinTech</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>International Conference in Venice - Artificial Intelligence, Financial Innovation and Credit Risk</t>
+          <t>37th Annual Conference of the Academy of Behavioral Finance &amp; Economics</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Venice, Italy</t>
+          <t>Santa Monica, California, USA</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>$99.00 USD</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Credit Risk and Advanced Analytics, Financial Innovation and Digital Transformation, Artificial Intelligence, Data Governance and Ethical Risk, Sustainability and Long-Term Value Creation, Systemic Risk, Resilience and Policy</t>
+          <t>Behavioral/Cognitive Finance &amp; Economics, Neuroscience/Neuromorphic Computing, Political Economy, Biological Anthropology, Brain-Computer Interfaces, Decision Making under risk and uncertainty, Venture Startups &amp; Exits, Investment &amp; Management, Entrepreneurship, Personal Finance, Behavioral Finance applications.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>36th Annual Conference on Financial Economics and Accounting (CFEA)</t>
+          <t>Colorado Finance Summit 2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-11-20</t>
+          <t>2026-12-10</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-11-21</t>
+          <t>2026-12-13</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Toronto, Ontario (Canada)</t>
+          <t>Vail, Colorado</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>100 CAD</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Financial economics and accounting</t>
+          <t>All areas of finance, theoretical and empirical contributions</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026 Lugano Real Estate and Urban Economics Conference</t>
+          <t>2026 UNSW Asset Pricing Workshop</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Lugano, Switzerland</t>
+          <t>Sydney (NSW, Australia)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0 AUD</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Real estate finance, urban economics, regional economics</t>
+          <t>All areas of Finance with a special focus on Asset Pricing</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Santiago Finance Workshop 2026</t>
+          <t>International Conference in Venice - Artificial Intelligence, Financial Innovation and Credit Risk</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-12-14</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-12-15</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Universidad de Chile, Diag. Paraguay 257, Santiago, Chile</t>
+          <t>Venice, Italy</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -782,71 +782,71 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Any topic in finance or financial economics</t>
+          <t>Credit Risk and Advanced Analytics, Financial Innovation and Digital Transformation, Artificial Intelligence, Data Governance and Ethical Risk, Sustainability and Long-Term Value Creation, Systemic Risk, Resilience and Policy</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>4th International Conference on Circular Economy, Business Strategy &amp; Management</t>
+          <t>36th Annual Conference on Financial Economics and Accounting (CFEA)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-11-20</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-11-21</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>EM Normandie Business School, Caen campus, France</t>
+          <t>Toronto, Ontario (Canada)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>100 CAD</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>sustainability, ESG, innovation, resilience, circular business models, future of management research</t>
+          <t>Financial economics and accounting</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Climate Finance &amp; Sustainability Conference</t>
+          <t>2026 Lugano Real Estate and Urban Economics Conference</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Lugano, Switzerland</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -856,34 +856,34 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Strategy and management, Accounting and finance, Entrepreneurship and innovation, Marketing and responsible consumption, Supply chain and operations management</t>
+          <t>Real estate finance, urban economics, regional economics</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>China Accounting and Finance Review (CAFR) Special Issue Conference 2026</t>
+          <t>Santiago Finance Workshop 2026</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2026-12-14</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-11-29</t>
+          <t>2026-12-15</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Zhongnan University of Economics and Law, Wuhan, China</t>
+          <t>Universidad de Chile, Diag. Paraguay 257, Santiago, Chile</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -893,71 +893,47 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>ESG in the AI Era: Challenges and Opportunities, AI-Driven ESG Reporting and Assurance, Algorithmic Bias, Ethics, and Fairness in ESG Analytics, Regulatory Responses to AI-Enabled ESG Practices, AI, Greenwashing, and Corporate Accountability, AI for Sustainable Finance and Investment Decision-Making</t>
+          <t>Any topic in finance or financial economics</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026 FMA Asia/Pacific Conference</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>2026-12-02</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>2026-12-04</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Massey University, Auckland, New Zealand</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>$50 USD (FMA-members), $60 USD (non-members)</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Financial decision-making, financial management, related topics</t>
-        </is>
-      </c>
+          <t>Please provide the text of the announcement so I can extract the required information.</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sixth Biennial Conference on Auto Lending</t>
+          <t>Climate Finance &amp; Sustainability Conference</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Federal Reserve Bank of Philadelphia</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -967,34 +943,34 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Auto lending and consumer finance, consumer demand and vehicle choice, loan pricing and contract design, underwriting and credit risk modeling, dealer intermediation and markups, borrower outcomes and delinquency dynamics, fraud and identity risk, fair lending and consumer compliance, subprime and near-prime market structure, repossession and loss mitigation, servicing and collections, alternative data and automated decisioning, electric vehicles and evolving collateral risk, used vehicle prices and depreciation, auto insurance interactions, fintech and market structure, auto asset-backed securities, spillovers from monetary policy and macroeconomic shocks.</t>
+          <t>Multi-stakeholder governance of sustainability initiatives, Managing business impacts on planetary boundaries, Inter- and intra-connectivity of environmental, social, and governance (ESG) factors, From disclosure to decision-usefulness in sustainability reporting, Regulatory competition in sustainability reporting and standard setting, ESG, sustainability, and climate finance, The role of artificial intelligence in advancing business sustainability, Design, scaling, and diffusion of sustainable business models, Social entrepreneurship and impact-driven ventures, Multi-dimensional sustainability claims and brand perceptions/performance, Stakeholder responses to corporate sustainability communication, Responsible consumption and consumer engagement in the circular economy, Operational resilience in the context of natural disasters and climate change, Technology adoption and implementation in sustainable supply chain management, Scope 3 emissions: measurement and management across the supply chain</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Frontiers in Machine Learning and Economics: Methods and Applications</t>
+          <t>China Accounting and Finance Review (CAFR) Special Issue Conference 2026</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-11-28</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-11-29</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Federal Reserve Bank of Philadelphia</t>
+          <t>Zhongnan University of Economics and Law, Wuhan, China</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1004,66 +980,66 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Methodological advances in analyzing complex and high-dimensional data sets; Methodological advances in natural language processing, particularly with respect to causal inference; Innovative applications of generative AI; The societal impacts of AI and algorithmic decision-making</t>
+          <t>ESG in the AI Era: Challenges and Opportunities, AI-Driven ESG Reporting and Assurance, Algorithmic Bias, Ethics, and Fairness in ESG Analytics, Regulatory Responses to AI-Enabled ESG Practices, AI, Greenwashing, and Corporate Accountability, AI for Sustainable Finance and Investment Decision-Making</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Workshop on Innovations in Credit Scoring</t>
+          <t>2026 FMA Asia/Pacific Conference</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-12-02</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Virtual</t>
+          <t>Massey University, Auckland, New Zealand</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>$50 USD (FMA-members), $60 USD (non-members)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Innovations in credit scoring, alternative data, fairness, transparency, data privacy, artificial intelligence, machine learning</t>
+          <t>Financial decision-making, financial management, related topics</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026 Conference on Real-Time Data Analysis, Methods, and Applications</t>
+          <t>Sixth Biennial Conference on Auto Lending</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1078,34 +1054,34 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>monitoring and forecasting of economic and financial developments, high-frequency data, survey data, text as data, transactions data, granular data, preliminary and revised data in economic policy formulation and analysis, machine learning applications in real-time macroeconomics, probabilistic forecasts and assessments of crisis risks, innovative data sets and toolboxes, seasonal and cyclical adjustment for real-time monitoring and forecasting</t>
+          <t>Auto lending, consumer finance, consumer demand and vehicle choice, loan pricing and contract design, underwriting and credit risk modeling, dealer intermediation and markups, borrower outcomes and delinquency dynamics, fraud and identity risk, fair lending and consumer compliance, subprime and near-prime market structure, repossession and loss mitigation, servicing and collections, role of alternative data and automated decisioning, electric vehicles and evolving collateral risk, used vehicle prices and depreciation, auto insurance interactions, fintech and market structure, auto asset-backed securities, spillovers from monetary policy and macroeconomic shocks.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026 Jacobs Levy Center Frontiers in Quantitative Finance Conference</t>
+          <t>Frontiers in Machine Learning and Economics: Methods and Applications</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2023-07-12</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Philadelphia, PA</t>
+          <t>Federal Reserve Bank of Philadelphia</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1115,51 +1091,51 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Quantitative methods and asset pricing</t>
+          <t>Methodological advances in analyzing complex and high-dimensional data sets, Methodological advances in natural language processing, particularly with respect to causal inference, Innovative applications of generative AI, The societal impacts of AI and algorithmic decision-making</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>34th Annual PBFEAM and 20th NYCU International conferences</t>
+          <t>Workshop on Innovations in Credit Scoring</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>National Yang Ming Chiao Tung University, Hsinchu, Taiwan</t>
+          <t>Virtual</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>USD $250 for On-line Presenter &amp; USD $300 for On-site Presenter</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Innovations in credit scoring, alternative data, fairness, transparency, data privacy, artificial intelligence, machine learning</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026 AIM Investment Conference</t>
+          <t>2026 Conference on Real-Time Data Analysis, Methods, and Applications</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1179,44 +1155,44 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Austin, Texas</t>
+          <t>Federal Reserve Bank of Philadelphia</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>$75 USD</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>mutual funds, hedge funds, pension funds, investment management</t>
+          <t>monitoring and forecasting of economic and financial developments, machine learning applications in real-time macroeconomics, probabilistic forecasts and assessments of crisis risks, using preliminary and revised data in economic policy formulation and analysis, related innovative data sets and toolboxes, seasonal and cyclical adjustment for real-time monitoring and forecasting</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026 Wharton Conference on Liquidity and Financial Fragility</t>
+          <t>2026 Jacobs Levy Center Frontiers in Quantitative Finance Conference</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>University of Pennsylvania, Philadelphia, PA</t>
+          <t>Philadelphia, PA</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1226,108 +1202,108 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Coordination failures, self-fulfilling beliefs, and runs; Fragility in banks and non-bank institutions; Liquidity and frictions in financial markets and macroeconomy; Systemic risk and financial regulation; Monetary policy and financial stability; Artificial intelligence (AI) and its implications for financial macroeconomic stability; The rise and potential risks in private credit markets; New payment technologies, stablecoins, tokenization, and their financial stability implications; Geopolitical tensions, trade conflicts, currency competition, and financial fragility; Inflation, interest rate risks, and implications on financial fragility; The real impact of crises and fragility on firms’ financing and investment policies</t>
+          <t>quantitative methods and asset pricing</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Towards a New Synthesis in Islamic Finance: Law, Economics and Shari’ah</t>
+          <t>34th Annual PBFEAM and 20th NYCU International conferences</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-11-27</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-11-28</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Online Conference from Durham University, England, UK</t>
+          <t>National Yang Ming Chiao Tung University, Hsinchu, Taiwan</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>USD $250 for On-line Presenter &amp; USD $300 for On-site Presenter</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Islamic finance, financial innovation, regulatory oversight, governance mechanisms, economic development, sustainability, social equity, inclusive economic development</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>74th Meeting of the EURO Working Group for Commodities and Financial Modelling (EWGCFM)</t>
+          <t>2026 AIM Investment Conference</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2026-11-22</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026-11-24</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Casa de Campo, La Romana, Dominican Republic</t>
+          <t>Austin, Texas</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>$75 USD</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Asset Pricing, Corporate Finance, Banking and Financial Institutions, Commodities and Energy Markets, Financial Modelling and Econometrics, Blockchain and Cryptocurrencies, Derivatives and Risk Management, Market Microstructure, Sustainable Finance</t>
+          <t>mutual funds, hedge funds, pension funds, investment management</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>FIRN 2026 ANU Money, Credit, and Financial Stability Meeting</t>
+          <t>2026 Wharton Conference on Liquidity and Financial Fragility</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Australian National University (ANU), Canberra, Australia</t>
+          <t>University of Pennsylvania, Philadelphia, PA</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1337,34 +1313,34 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Monetary policy and transmission mechanisms, Credit markets and financial intermediation, Banking, liquidity, and regulation, Financial crises and systemic risk, Macro-finance</t>
+          <t>Coordination failures, self-fulfilling beliefs, and runs; Fragility in banks and non-bank institutions; Liquidity and frictions in financial markets and macroeconomy; Systemic risk and financial regulation; Monetary policy and financial stability; Artificial intelligence (AI) and its implications for financial macroeconomic stability; The rise and potential risks in private credit markets; New payment technologies, stablecoins, tokenization, and their financial stability implications; Geopolitical tensions, trade conflicts, currency competition, and financial fragility; Inflation, interest rate risks, and implications on financial fragility; The real impact of crises and fragility on firms’ financing and investment policies</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Chicago Fed/University of Chicago Conference on Municipal Bond Markets</t>
+          <t>Towards a New Synthesis in Islamic Finance: Law, Economics and Shari’ah</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Federal Reserve Bank of Chicago</t>
+          <t>Online Conference from Durham University, England, UK</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1374,34 +1350,34 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Unpublished and highly policy-relevant research papers on municipal bond markets, primary market frictions, secondary market frictions, the role of retail investors, government policies targeting investors for bond price formation, state and federal policies on state and local government access to external finance</t>
+          <t>Islamic law and finance, financial innovation, regulatory oversight, governance mechanisms, economic development, sustainability, social equity, inclusive economic development</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Inaugural Annual Conference on Insurance</t>
+          <t>74th Meeting of the EURO Working Group for Commodities and Financial Modelling (EWGCFM)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-11-22</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-11-24</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Federal Reserve Bank of Chicago</t>
+          <t>Casa de Campo, La Romana, Dominican Republic</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1411,34 +1387,34 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>life insurance, Property &amp; Casualty insurance, reinsurance and risk transfer, mergers and other ownership changes, private equity ownership and impact on industry, indexed and variable annuities, household insurance choices, insurances’ investment and funding strategies, catastrophe risk, impact of insurance regulation</t>
+          <t>Asset Pricing, Corporate Finance, Banking and Financial Institutions, Commodities and Energy Markets, Financial Modelling and Econometrics, Blockchain and Cryptocurrencies, Derivatives and Risk Management, Market Microstructure, Sustainable Finance</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Payments, Digital Assets, AI and the Future of Financial Markets</t>
+          <t>FIRN 2026 ANU Money, Credit, and Financial Stability Meeting</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Imperial Business School, London</t>
+          <t>Australian National University (ANU), Canberra, Australia</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1448,34 +1424,34 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Digital platforms, banking, and financial intermediation; Artificial intelligence, machine learning, and financial decision-making; Blockchain, tokenization, digital assets, and decentralized finance; Payment systems, central bank digital currencies, and stablecoins; FinTech regulation, supervision, market design, and financial stability; Data, privacy, cybersecurity, and consumer protection in finance; Entrepreneurial finance, venture capital, and innovation in financial services; Household finance, inclusion, and welfare effects of financial technology; Market microstructure, trading technologies, and liquidity; Competition between banks, platforms, and non-bank financial institutions</t>
+          <t>Monetary policy and transmission mechanisms, Credit markets and financial intermediation, Banking, liquidity, and regulation, Financial crises and systemic risk, Macro-finance</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026 Conference on Auditing and Capital Markets</t>
+          <t>Inaugural Annual Conference on Insurance</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Washington, DC</t>
+          <t>Federal Reserve Bank of Chicago</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1485,34 +1461,34 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Audit-related topics, economic impact of auditing, audit regulation, audit oversight</t>
+          <t>Reinsurance and risk transfer, Mergers and other ownership changes, Private equity ownership and impact on industry, Indexed, variable annuities and other savings products, Household insurance choices, Insurances’ investment and funding strategies, Catastrophe risk, Impact of insurance regulation</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026 Future Scholars in Finance Forum</t>
+          <t>Payments, Digital Assets, AI and the Future of Financial Markets</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Beijing, China</t>
+          <t>Imperial Business School, London</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1522,34 +1498,34 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>All areas of finance</t>
+          <t>Digital platforms, banking, and financial intermediation; Artificial intelligence, machine learning, and financial decision-making; Blockchain, tokenization, digital assets, and decentralized finance; Payment systems, central bank digital currencies, and stablecoins; FinTech regulation, supervision, market design, and financial stability; Data, privacy, cybersecurity, and consumer protection in finance; Entrepreneurial finance, venture capital, and innovation in financial services; Household finance, inclusion, and welfare effects of financial technology; Market microstructure, trading technologies, and liquidity; Competition between banks, platforms, and non-bank financial institutions</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Prototypes for Humanity 2026 Short Papers Platform</t>
+          <t>2026 Conference on Auditing and Capital Markets</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-11-15</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Dubai, UAE</t>
+          <t>Washington, DC</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1559,34 +1535,34 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Wellbeing and Human Performance, Infrastructures and Cities, Autonomous Systems and Advanced Manufacturing, Environment, Sustainability and Energy, Mobility and Logistics, Socio-Economic Empowerment, Digital Economies and Future Markets, Open and Speculative</t>
+          <t>Audit-related topics, economic impact of auditing, audit regulation, audit oversight</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>15th LaBS International Banking Workshop</t>
+          <t>Future Scholars in Finance Forum</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>HSE University and online</t>
+          <t>Beijing, China</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1596,34 +1572,34 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Banking in Emerging Markets, Household finance</t>
+          <t>All areas of finance</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026 Federal Reserve Stress Testing Research Conference</t>
+          <t>Prototypes for Humanity 2026 Short Papers Platform</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2026-11-05</t>
+          <t>2026-11-15</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Boston, Massachusetts</t>
+          <t>Dubai, UAE</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1633,71 +1609,71 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Economic and macroprudential effects of stress tests and bank regulation, novel approaches to modeling bank profitability, financial risks, and operational risks, design and applications of stress scenarios and reverse stress testing, nonbank credit intermediation, financial instruments for risk transfer, recent developments in bank regulation, impact of emerging technologies on banks and their regulators</t>
+          <t>Wellbeing and Human Performance, Infrastructures and Cities, Autonomous Systems and Advanced Manufacturing, Environment, Sustainability and Energy, Mobility and Logistics, Socio-Economic Empowerment, Digital Economies and Future Markets, Open and Speculative</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>EUROFIDAI-ESSEC Paris December Finance Meeting</t>
+          <t>15th LaBS International Banking Workshop</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2026-12-17</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026-12-17</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Pullman Paris Montparnasse Hotel</t>
+          <t>HSE University and online</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>75€</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>All areas of finance</t>
+          <t>Banking in Emerging Markets: Challenges and Opportunities, theoretical and empirical research in Banking or Household finance</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>EBA's 15th Policy Research Workshop</t>
+          <t>2026 Federal Reserve Stress Testing Research Conference</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2026-11-18</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>EBA premises (Paris, France) and remotely</t>
+          <t>Boston, Massachusetts</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1707,34 +1683,34 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Competitiveness and efficiency in the prudential rulebook without undermining resilience; Impacts of efficiency and proportionality; Competition, innovation, market entry, cross border growth and new areas under financial supervision; Proportionate integration of ESG risks in governance, strategy, and remuneration frameworks</t>
+          <t>The economic and macroprudential effects of stress tests and bank regulation; Novel approaches to modeling bank profitability, financial risks, and operational risks; Design and applications of stress scenarios and reverse stress testing; Nonbank credit intermediation; Financial instruments for risk transfer; Recent developments in bank regulation; The impact of emerging technologies on banks and their regulators</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>3rd Financial Fraud, Misconduct and Market Manipulation Conference</t>
+          <t>EBA's 15th Policy Research Workshop</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-11-18</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Lancaster University, England</t>
+          <t>EBA premises (Paris, France) and remotely</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1744,34 +1720,34 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Theoretical and empirical analysis of financial fraud, case studies of recent instances of market misconduct, insider trading, implications of financial fraud/market manipulation for market efficiency, stability, and asset pricing, market manipulation at a high-frequency (intraday) level, fraudulent activities and cryptocurrency markets, social networks, fake news and their effect on financial markets, money laundering and banking, conflicts of interest and their implications for various stakeholders and financial markets, hedge funds/mutual funds and their involvement in market misconduct, statistical/machine learning methods for fraud detection, cyber security and cyber risk management, regulatory response to financial misconduct, unintended consequences of politics and regulations</t>
+          <t>Competitiveness and efficiency in the prudential rulebook without undermining resilience, impacts of efficiency and proportionality, competition, innovation, market entry, cross border growth and new areas under financial supervision, proportionate integration of ESG risks in governance, strategy, and remuneration frameworks</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>22nd Annual Haskell &amp; White Corporate Reporting and Governance Conference</t>
+          <t>Financial Fraud, Misconduct and Market Manipulation Conference</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>California State University, Fullerton</t>
+          <t>Lancaster University, England</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1781,34 +1757,34 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>All areas of accounting and finance, including interdisciplinary research related to corporate reporting, governance, and financial markets</t>
+          <t>Theoretical and empirical analysis of financial fraud, Case studies of recent instances of market misconduct, Insider trading, Implication of financial fraud/market manipulation for market efficiency, stability, and asset pricing, Market manipulation at a high-frequency (intraday) level, Fraudulent activities and crypto currency markets, Social networks, fake news, and their effect on financial markets, Money laundering and banking, Conflicts of interests and their implications for various stakeholders and financial markets, Hedge funds/Mutual funds and their involvement in market misconduct, Statistical/ Machine Learning methods for fraud detection, Cyber security and cyber risk management, Regulatory response to financial misconduct, Unintended consequences of politics and regulations</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>25th Annual Bank Research Conference</t>
+          <t>22nd Annual Haskell &amp; White Corporate Reporting and Governance Conference</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Arlington, VA</t>
+          <t>California State University, Fullerton</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1818,108 +1794,108 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Regulatory reform options and considerations, Risk and resiliency in the financial system, Real effects of financial turmoil, Innovations in financial intermediation, Deposit insurance and stability, Emerging competitive threats to traditional banking, AI and technology in finance, Banks’ role in the 21st Century</t>
+          <t>All areas of accounting and finance, interdisciplinary research related to corporate reporting, governance, and financial markets</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>The Future of Decision-Making and Risk-Taking: Bridging Finance, Economics, Brain, and Behavior</t>
+          <t>25th Annual Bank Research Conference</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Santa Monica, California, USA</t>
+          <t>Arlington, VA</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>$99.00 USD</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Behavioral/Cognitive Finance &amp; Economics, Neuroscience/Neuromorphic Computing, Political Economy, Biological Anthropology, Brain-Computer Interfaces, Development of New Financial &amp; Economic Models, Decision Making under conditions of risk and uncertainty, Venture Startups &amp; Exits, Markets &amp; Capital, Investment &amp; Management, Entrepreneurship, Innovation, Economic Development, Sustainable Finance, Personal Finance, Teaching, Learning, and Training using AI or AGI, Empirical Works, Evidence-Based Financial and Retirement Planning Best Practices, Behavioral/Cognitive Value Investing.</t>
+          <t>Regulatory reform options and considerations, Risk and resiliency in the financial system, Real effects of financial turmoil, Innovations in financial intermediation, Deposit insurance and stability, Emerging competitive threats to traditional banking, AI and technology in finance, Banks’ role in the 21st Century</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>17th Emerging Markets Conference</t>
+          <t>The Future of Decision-Making and Risk-Taking: Bridging Finance, Economics, Brain, and Behavior</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2026-12-13</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Mumbai, India</t>
+          <t>Santa Monica, California, USA</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>$99.00 USD</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>The sources of economic success or failure in EMs; Finance in EMs; Political economy, law, public administration, regulation in EMs; The impact of populism upon sustained growth; Insights into large EMs; Insights from narrow research projects; The new phase of globalization; Features of a society that enable or disable convergence; Grand challenges such as climate change; State capability in EMs; The interplay of military affairs, foreign policy and economics for EMs</t>
+          <t>Behavioral/Cognitive Finance &amp; Economics, Neuroscience/Neuromorphic Computing, Political Economy, Biological Anthropology, Brain-Computer Interfaces, Development of New Financial &amp; Economic Models, Decision Making under risk and uncertainty, Venture Startups &amp; Exits, Financial/Capital Markets, Investment &amp; Management, Entrepreneurship, Personal Finance, Pedagogy, Behavioral Finance in Practice</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026 International Forum on Financial Regulation and RegTech</t>
+          <t>17th Emerging Markets Conference</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-12-13</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-12-16</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Beihang University, Beijing, China</t>
+          <t>Mumbai, India</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -1929,14 +1905,14 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Financial regulation, Regulatory Technology (RegTech), FinTech, financial security, algorithmic bias, data privacy, financial fraud detection, systemic financial risk, AI applications in finance, and risk assessment methodologies.</t>
+          <t>The sources of economic success or failure in EMs, Finance in EMs (households, financial markets, financial intermediaries, firms and finance, finance and growth), Political economy, law, public administration, regulation in EMs, The impact of populism upon the possibility of sustained growth, Insights into large EMs that matter in and of themselves, Insights from narrow research projects that illuminate EMs in general, The new phase of globalisation and its consequences for international trade, international finance and the nature of the EM firm, Features of a society that enable or disable convergence into the “normal” package of high levels of freedom and prosperity, The puzzles faced by all kinds of decision makers: individuals, civil society actors, firms, all levels of government, Grand challenges such as climate change: implications for EMs and ramifications of choices made in EMs, State capability in EMs, The interplay of military affairs, foreign policy and economics for EMs</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026 International Symposium on Climate, Finance, and Sustainability (ISCFS-2026)</t>
+          <t>2026 International Forum on Financial Regulation and RegTech</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1946,17 +1922,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>House of Management Science, Paris Pantheon-Assas University, 1 rue Guy-de-la-Brosse 75005 Paris, France</t>
+          <t>Beihang University, Beijing, China</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -1966,108 +1942,108 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Carbon Finance and Taxes, Climate and Economic Modeling in Policy Making, Climate Finance, Climate Negotiations and Scenarios, Climate Risk and Disclosures, Climate-resilient Economies, Energy Derivatives: Pricing and Hedging, Energy Markets: Modeling and Forecasting, Energy, Environment, and Climate Models, Financial and Economic Analysis of Energy Markets, Financial Regulation of Energy and Environmental Markets, Green Finance and Sustainable Investment, Just Energy Transition, Macroeconomic Implications of Net-Zero Carbon Emissions, Nature-based Financial Instruments for Climate Change Mitigation, Natural Resources, Risk, Welfare, and Social Preferences, Renewable Energy, Regulation and Energy Governance, Role of Financial Institutions in Sustainability</t>
+          <t>Financial Regulation &amp; RegTech Innovation, Risk Assessment &amp; Management, AI, LLMs &amp; Financial Infrastructure</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>5th Annual Academic - 2026 DeFi &amp; Digital Currencies Conference</t>
+          <t>2026 International Symposium on Climate, Finance, and Sustainability (ISCFS-2026)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>The Shard, London, UK</t>
+          <t>House of Management Science, Paris Pantheon-Assas University, 1 rue Guy-de-la-Brosse 75005 Paris, France</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>£45</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>DeFi Protocols, Lending and Borrowing Protocols, Decentralized Exchanges (DEXs), Blockchain Economics, Stablecoins and CBDCs, Digital Money and Payments, Tokenisation of real-world assets, Traditional and Decentralized Finance Interaction, Digital Finance and Inclusion</t>
+          <t>Carbon Finance and Taxes, Climate and Economic Modeling in Policy Making, Climate Finance, Climate Negotiations and Scenarios, Climate Risk and Disclosures, Climate-resilient Economies, Energy Derivatives: Pricing and Hedging, Energy Markets: Modeling and Forecasting, Energy, Environment, and Climate Models, Financial and Economic Analysis of Energy Markets, Financial Regulation of Energy and Environmental Markets, Green Finance and Sustainable Investment, Just Energy Transition, Macroeconomic Implications of Net-Zero Carbon Emissions, Nature-based Financial Instruments for Climate Change Mitigation, Natural Resources, Risk, Welfare, and Social Preferences, Renewable Energy, Regulation and Energy Governance, Role of Financial Institutions in Sustainability</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>3rd Arne Ryde Conference on Crypto, Fintech and Payments</t>
+          <t>5th Annual Academic - 2026 DeFi &amp; Digital Currencies Conference</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Lund, Sweden</t>
+          <t>The Shard, London, UK</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>£45</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Crypto and blockchain technology, Crypto markets, households, and the real economy, Environmental and social impact of crypto markets, Interaction between traditional finance and decentralized finance, Stablecoins, Central Bank Digital Currencies (CBDCs), Financial technology (Fintech), Payment systems, Open banking and data sharing, Digital tools in financial services, Financial inclusion, development, and welfare in digital finance</t>
+          <t>DeFi Protocols, Lending and Borrowing Protocols, Decentralized Exchanges, Blockchain Economics, Stablecoins and CBDCs, Digital Money and Payments, Tokenisation of real-world assets, Traditional and Decentralized Finance Interaction, Digital Finance and Inclusion</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Institute for Quantitative Investment Research Autumn Residential Seminar 2026</t>
+          <t>3rd Arne Ryde Conference on Crypto, Fintech and Payments</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Ashdown Park Hotel &amp; Country Club, Wych Cross, East Sussex, UK</t>
+          <t>Lund, Sweden</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2077,34 +2053,34 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>New risks in a changing political environment, investment management excellence, innovative and high-quality research related to investment practitioners</t>
+          <t>Crypto and blockchain technology, Crypto markets, Environmental and social impact of crypto markets, Interaction between traditional finance and decentralized finance, Stablecoins, Central Bank Digital Currencies (CBDCs), Financial technology (Fintech), Payment systems, Open banking and data sharing, Digital tools in financial services, Financial inclusion, development, and welfare in digital finance</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>10th Shanghai-Edinburgh-London Finance Conference On Sustainable Finance in the Digital Era</t>
+          <t>Institute for Quantitative Investment Research Autumn Residential Seminar 2026</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Shanghai and online</t>
+          <t>Ashdown Park Hotel &amp; Country Club, Wych Cross, East Sussex, UK</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2114,34 +2090,34 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Financial development, financial inclusion, policy frameworks and regulatory challenges in sustainable finance, cross-border sustainable finance flows, corporate governance and greenwashing detection, ESG backlash and anti-ESG movements, AI and machine learning applications in ESG, big data and natural language processing for ESG, blockchain applications in carbon markets and green bonds, digital finance and decentralised finance in low-carbon transition, fintech-enabled green lending and climate insurance</t>
+          <t>New risks in a changing political environment, innovative research related to investment management</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>22nd Annual Conference of the Asia-Pacific Association of Derivatives</t>
+          <t>10th Shanghai-Edinburgh-London Finance Conference On Sustainable Finance in the Digital Era</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Park Hyatt Busan, Busan, Korea</t>
+          <t>Shanghai and online</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2151,182 +2127,182 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Derivatives; Volatility; Risk Management; Asset Pricing; Investments; Corporate Finance; Market Microstructure; Fintech; Regulation; Behavioral Finance</t>
+          <t>Financial development, financial inclusion, and their role in sustainable economic growth; Policy frameworks and regulatory challenges shaping sustainable finance adoption in developed and emerging markets; Cross-border sustainable finance flows and international regulatory coordination; Corporate governance, greenwashing detection, and market responses to ESG commitments; ESG backlash, anti-ESG movements, and the political economy of sustainable finance; AI and machine learning applications in ESG investment strategies, sustainability disclosure, and climate risk modelling; Big data and natural language processing in measuring and monitoring ESG performance; Blockchain applications in carbon markets, green bonds, and regulatory compliance; Digital finance, decentralised finance (DeFi), and emerging technologies in supporting a low-carbon transition; Fintech-enabled green lending, climate insurance, and impact investing</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>FIRN Melbourne Asset Pricing Meeting</t>
+          <t>22nd Annual Conference of the Asia-Pacific Association of Derivatives</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Melbourne, Australia</t>
+          <t>Busan, Korea</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>0 AUD</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Theoretical and empirical models of asset prices and returns, return predictability, empirical methodology, macro-finance, the study of financial institutions as related to asset prices, information and liquidity in asset markets, behavioural investment studies, asset market structure and microstructure, risk analysis, hedge funds, mutual funds, pension funds, ESG, and alternative investments.</t>
+          <t>Derivatives; Volatility; Risk Management; Asset Pricing; Investments; Corporate Finance; Market Microstructure; Fintech; Regulation; Behavioral Finance</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Johns Hopkins Carey Finance Conference</t>
+          <t>FIRN Melbourne Asset Pricing Meeting</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Johns Hopkins Carey Business School, 100 International Drive, Baltimore, MD</t>
+          <t>Melbourne, Australia</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0 AUD</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>All areas of finance, particularly early-stage papers that would benefit from feedback and discussion</t>
+          <t>theoretical and empirical models of asset prices and returns, return predictability, empirical methodology, macro-finance, the study of financial institutions as related to asset prices, information and liquidity in asset markets, behavioural investment studies, asset market structure and microstructure, risk analysis, hedge funds, mutual funds, pension funds, ESG, and alternative investments</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>5th Holden Conference in Finance and Real Estate</t>
+          <t>Johns Hopkins Carey Finance Conference</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Bloomington, IN</t>
+          <t>Johns Hopkins Carey Business School, 100 International Drive, Baltimore, MD</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>$95 USD</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Empirical and theoretical papers in all finance and real estate areas</t>
+          <t>All areas of finance, particularly early-stage papers</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>12th P2P Financial Systems International Workshop (P2PFISY 2026)</t>
+          <t>5th Holden Conference in Finance and Real Estate</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Astana, Kazakhstan</t>
+          <t>Bloomington, IN</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>$95 USD</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Regulation &amp; Compliance in Digital Asset Markets, Fraud, Financial Crime &amp; Forensics in Crypto Markets, CBDCs and Digital Public Infrastructure, Stablecoins and Digital Payment Systems, Artificial Intelligence in Financial Systems, Consumer Protection, Data Governance, and Trust in Digital Finance, Tokenisation of Real-World Assets (RWA)</t>
+          <t>empirical and theoretical papers in all finance and real estate areas</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026 New Zealand Finance Meeting</t>
+          <t>12th P2P Financial Systems International Workshop (P2PFISY 2026)</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2026-12-14</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Auckland, New Zealand</t>
+          <t>Astana, Kazakhstan</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2336,182 +2312,182 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>All topics related to the field of finance</t>
+          <t>Regulation &amp; Compliance in Digital Asset Markets, Fraud, Financial Crime &amp; Forensics in Crypto Markets, CBDCs and Digital Public Infrastructure, Stablecoins and Digital Payment Systems, Artificial Intelligence in Financial Systems, Consumer Protection, Data Governance, and Trust in Digital Finance, Tokenisation of Real-World Assets (RWA)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026 Annual Community Bank Research Conference</t>
+          <t>2026 New Zealand Finance Meeting</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-12-14</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-12-16</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Federal Reserve Bank of St. Louis in St. Louis, MO</t>
+          <t>Auckland, New Zealand</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>0 USD</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>The role of community banks in the U.S. financial system, impact of community banks on local/state economic activity, community banks’ response to financial and economic shocks, effects of regulatory policy on community banks, challenges and opportunities faced by community banks, advantages and disadvantages of the community bank business model</t>
+          <t>All topics related to the field of finance</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Stigler Center-CEPR Political Economy of Finance Conference 2026: Crony Capitalism in 21st Century America</t>
+          <t>2026 Annual Community Bank Research Conference</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Gleacher Center - Chicago</t>
+          <t>Federal Reserve Bank of St. Louis in St. Louis, MO</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0 USD</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Crony capitalism in 21st century America, political economy, business and political elite interactions, economic power and political influence</t>
+          <t>The role of community banks in the U.S. financial system, impact of community banks on local/state economic activity, community banks’ response to financial and economic shocks, effects of regulatory policy on community banks, challenges and opportunities faced by community banks, advantages and disadvantages of the community bank business model</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>15th Fixed Income and Financial Institutions (FIFI) Conference</t>
+          <t>Stigler Center-CEPR Political Economy of Finance Conference 2026: Crony Capitalism in 21st Century America</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2026-10-31</t>
+          <t>2026-11-07</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>University of South Carolina in Columbia, SC</t>
+          <t>Gleacher Center - Chicago</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>75 USD</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>fixed income, commercial and investment banks, asset management and mutual fund companies, short sellers, hedge funds, broker-dealers, insurance companies</t>
+          <t>Crony capitalism in 21st century America, political economy, business and political elite dynamics</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Higher Education Finance Research Conference</t>
+          <t>15th Fixed Income and Financial Institutions (FIFI) Conference</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Federal Reserve Bank of Philadelphia</t>
+          <t>University of South Carolina in Columbia, SC</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>75 USD</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>financial aid, student debt, higher education finance</t>
+          <t>fixed income, commercial and investment banks, asset management, mutual fund companies, short sellers, hedge funds, broker-dealers, insurance companies</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Wharton–Chicago–Harvard Insolvency and Restructuring Conference (WCHIRC)</t>
+          <t>Higher Education Finance Research Conference</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>University of Pennsylvania, Philadelphia, PA</t>
+          <t>Federal Reserve Bank of Philadelphia</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2521,34 +2497,34 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Corporate financial distress and bankruptcy, Liability management and out-of-court restructurings, Chapter 11 and formal reorganization processes, Consumer bankruptcy, Leveraged lending and private credit, Creditor governance and capital structure dynamics, Distressed debt markets and asset pricing, Financial contracting and covenant design, Bankruptcy law, courts, and institutional design, Operational restructuring and firm performance</t>
+          <t>financial aid, student debt, higher education finance</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Financial Decision-Making Conference 2026</t>
+          <t>2026 Wharton–Chicago–Harvard Insolvency and Restructuring Conference (WCHIRC)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Bozeman, MT</t>
+          <t>University of Pennsylvania, Philadelphia, PA</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2558,34 +2534,34 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>household finance, financial literacy and education, consumer financial behavior, retirement and savings decisions, financial education interventions, fintech and digital finance, financial advice and delegation, debt and credit decisions, insurance decisions, behavioral finance, financial inclusion</t>
+          <t>Corporate financial distress and bankruptcy, Liability management and out-of-court restructurings, Chapter 11 and formal reorganization processes, Consumer bankruptcy, Leveraged lending and private credit, Creditor governance and capital structure dynamics, Distressed debt markets and asset pricing, Financial contracting and covenant design, Bankruptcy law, courts, and institutional design, Operational restructuring and firm performance</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>39th Australasian Finance and Banking Conference</t>
+          <t>Financial Decision-Making Conference 2026</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2026-12-10</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>2026-12-12</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Sydney, Australia</t>
+          <t>Bozeman, MT</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2595,145 +2571,145 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Opportunities and Risks of AI Technology in Finance, CBDCs, Fintech, and Digital Finance, Sustainable Investment</t>
+          <t>household finance, financial literacy and education, consumer financial behavior, retirement and savings decisions, financial education interventions, fintech and digital finance, financial advice and delegation, debt and credit decisions, insurance decisions, behavioral finance, and financial inclusion</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Finance and Real Estate Conference 2026</t>
+          <t>39th Australasian Finance and Banking Conference</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-12-10</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-12-12</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Miami University, Oxford, OH</t>
+          <t>Sydney, Australia</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>$50 USD</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Asset pricing and valuation, Corporate finance, Real estate markets and investment, Risk management and financial regulation, Urban economics and housing policy, Sustainable and green finance, Behavioral finance</t>
+          <t>Opportunities and Risks of AI Technology in Finance, CBDCs, Fintech, and Digital Finance, Sustainable Investment</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>UGA Fall Finance Conference 2026</t>
+          <t>Finance and Real Estate Conference 2026</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Athens, GA</t>
+          <t>Miami University, Oxford, OH</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>70 USD</t>
+          <t>$50 USD</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>All areas of finance</t>
+          <t>Asset pricing and valuation, Corporate finance, Real estate markets and investment, Risk management and financial regulation, Urban economics and housing policy, Sustainable and green finance, Behavioral finance</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Inquire Europe Autumn Conference: “Expectations and Asset Prices”</t>
+          <t>UGA Fall Finance Conference 2026</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Prague, Czech Republic</t>
+          <t>Athens, GA</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>70 USD</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>deviations from rational expectations and their implications; optimism and pessimism in asset valuations and market dynamics; investment strategies and anomalies; factor investing; strategic and tactical asset allocation; portfolio choice under model and parameter uncertainty; and short selling</t>
+          <t>All areas of finance</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>WFE’s Sustainability Conference 2026</t>
+          <t>Inquire Europe Autumn Conference: “Expectations and Asset Prices”</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Luxembourg</t>
+          <t>Prague, Czech Republic</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -2743,108 +2719,108 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Transition finance and market design, Regulatory fragmentation and divergence, Sustainability reporting, data and assurance, Nature and biodiversity in capital markets, Just transition, social and gender finance, Proportionality for SMEs and emerging markets, Carbon market architecture</t>
+          <t>Expectations and Asset Prices, deviations from rational expectations, optimism and pessimism in asset valuations, investment strategies and anomalies, factor investing, strategic and tactical asset allocation, portfolio choice under model and parameter uncertainty, short selling, institutional investing and asset management</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026 FMA Annual Meeting</t>
+          <t>WFE’s Sustainability Conference 2026</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Tampa, FL</t>
+          <t>Luxembourg</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>$75 (current FMA members); $85 (non-members)</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Financial decision-making, financial management, all areas of finance</t>
+          <t>Transition finance and market design; Regulatory fragmentation and divergence; Sustainability reporting, data and assurance; Nature and biodiversity in capital markets; Just transition, social and gender finance; Proportionality for SMEs and emerging markets; Carbon market architecture</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>AI in Finance Conference</t>
+          <t>2026 FMA Annual Meeting</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Montréal, QC, Canada</t>
+          <t>Tampa, FL</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>$75 (current FMA members); $85 (non-members)</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Machine learning and artificial intelligence in asset pricing and financial econometrics; Portfolio management, trading strategies, and risk management using AI; Large language models (LLMs), NLP, and textual analysis in finance; Corporate finance applications including M&amp;A and investment decisions; Banking, credit markets, and financial intermediation; Cryptocurrency, digital assets, and decentralized finance; ESG, sustainability, and climate finance; Financial regulation, policy analysis, and central bank communication; Real estate finance and urban economics; Alternative data and high-dimensional financial datasets; Investor behavior, sentiment, and attention; Macroeconomic and financial risk forecasting; AI in Sustainability and Climate Finance; AI and Real Estate</t>
+          <t>All areas of finance, financial decision-making, financial management, research projects, results of work in progress, recently completed work.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026 Summer Research Conference</t>
+          <t>AI in Finance Conference 2026</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Indian School of Business, Hyderabad Campus</t>
+          <t>Montréal, QC, Canada</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -2854,34 +2830,34 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Recent Advances in Finance, corporate finance, asset pricing, behavioral finance, financial intermediation, household finance, market microstructure</t>
+          <t>Machine learning and artificial intelligence in asset pricing and financial econometrics, Portfolio management, trading strategies, and risk management using AI, Large language models (LLMs), NLP, and textual analysis in finance, Corporate finance applications including M&amp;A and investment decisions, Banking, credit markets, and financial intermediation, Cryptocurrency, digital assets, and decentralized finance, ESG, sustainability, and climate finance, Financial regulation, policy analysis, and central bank communication, Real estate finance and urban economics, Alternative data and high-dimensional financial datasets, Investor behavior, sentiment, and attention, Macroeconomic and financial risk forecasting</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>International Risk Management Conference 2026</t>
+          <t>2026 Summer Research Conference</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Warsaw, Poland</t>
+          <t>Indian School of Business, Hyderabad Campus</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -2891,34 +2867,34 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Asset pricing; Banking; Financial econometrics; Capital markets; Financial intermediation; Corporate finance; Financial crises; Corporate governance; Market microstructure; Financial regulation; International corporate finance; Risk management; Emerging market; Corporate investment decision; Global risk markets; Macro-financial linkages; Financial policy securitization; Behavioural finance; Financial integration; Mathematical &amp; computational finance; Stochastic optimization approaches in finance; Mergers &amp; acquisitions; Modelling, money and liquidity; Sustainable finance; Climate change risk; AI innovation; crypto and related assets and technology</t>
+          <t>Recent Advances in Finance, corporate finance, asset pricing, behavioral finance, financial intermediation, household finance, market microstructure</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Second USTC Frontiers in Finance Conference</t>
+          <t>International Risk Management Conference 2026</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>International Finance Institute, University of Science and Technology of China, No. 1789 Guangxi Road, Binhu New District, Hefei City, Anhui Province, P.R. China</t>
+          <t>Warsaw, Poland</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -2928,14 +2904,14 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>All topics of finance</t>
+          <t>Asset pricing; Banking; Financial econometrics; Capital markets; Financial intermediation; Corporate finance; Financial crises; Corporate governance; Market microstructure; Financial regulation; International corporate finance; Risk management; Emerging market; Corporate investment decision; Global risk markets; Macro-financial linkages; Financial policy securitization; Behavioural finance; Financial integration; Mathematical &amp; computational finance; Stochastic optimization approaches in finance; Mergers &amp; acquisitions; Modelling, money and liquidity; Sustainable finance; Climate change risk; AI innovation; crypto and related assets and technology</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Fischer-Shain Research Conference 2026</t>
+          <t>Second USTC Frontiers in Finance Conference</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2945,91 +2921,91 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Philadelphia, PA</t>
+          <t>International Finance Institute, University of Science and Technology of China, No. 1789 Guangxi Road, Binhu New District, Hefei City, Anhui Province, P.R. China</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>50 USD</t>
+          <t>0 CNY</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>financial intermediation, banking, and financial services</t>
+          <t>All topics of finance</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ECB Money Market Conference 2026</t>
+          <t>Fischer-Shain Research Conference 2026</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2026-11-05</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>European Central Bank, Frankfurt am Main, Germany</t>
+          <t>Philadelphia, PA</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>50 USD</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Money markets and monetary policy implementation, technological innovation in money markets such as stable coins, CBDCs, instant payments, functioning of money markets including roles of non-bank financial institutions and dealer intermediation, macroeconomic implications of short-term rate volatility and geopolitical developments</t>
+          <t>financial intermediation, banking, financial services</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Finance in the Digital Age (FiDA) Workshop</t>
+          <t>ECB Money Market Conference 2026</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Calgary, Canada</t>
+          <t>European Central Bank, Frankfurt am Main, Germany</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3039,34 +3015,34 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>AI, DeFi, robo-advisors, neurofinance, decentralized finance</t>
+          <t>Money markets and monetary policy implementation, money markets and technological innovation, functioning of money markets</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>7th LTI@UniTO/Bank of Italy Workshop on Long-term investors’ trends: theory and practice</t>
+          <t>Finance in the Digital Age (FiDA) Workshop</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Bank of Italy, Rome, Italy</t>
+          <t>Calgary, Canada</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3076,14 +3052,14 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Long-term investors’ strategies and behavior, long-term investors’ role in financing the real economy, shifting equilibria in government bond markets, sustainable investment strategies, challenges for long-term investors, non-bank investors in credit intermediation, rise of cryptocurrencies and fintech, emerging trends in asset allocation and risk management, shock transmission mechanisms, use of big data and AI in investment, innovations in financial markets, geopolitical risks, demographic transitions effects on financial markets.</t>
+          <t>AI, DeFi, robo-advisors, neurofinance</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>7th Annual RCF-ECGI Corporate Finance and Governance Conference</t>
+          <t>7th LTI@UniTO/Bank of Italy Workshop on Long-term investors’ trends: theory and practice</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3093,239 +3069,239 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Madrid, Spain, and virtually</t>
+          <t>Bank of Italy, Rome, Italy</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>€350 in person (for conference dinner, lunches, and coffee breaks), €50 online option (for administrative / tech support)</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>capital structure, corporate and securities law, corporate culture, corporate failure, corporate finance and public policy, corporate governance, corporate restructuring, corporate social responsibility, crowdfunding, dividends, payout policy, and repurchases, entrepreneurial finance, family business, financial contracting, financial intermediation, financial literacy, fintech, fraud, innovation, IPOs and SEOs, mergers and acquisitions, misconduct, private debt, private equity, trade credit, socially responsible investments, sustainable finance, real options, and venture capital</t>
+          <t>Long-term investors’ strategies and behavior, long-term investors’ role in financing the real economy, shifting equilibria in government bond markets, sustainable investment strategies, challenges for long-term investors, non-bank investors in credit intermediation, rise of cryptocurrencies and fintech, asset allocation and risk management trends, shock transmission mechanisms, use of big data and AI in investment processes, innovations in financial markets, geopolitical risks, effects of demographic transitions on financial markets.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Fintech and Financial Institutions Research Conference</t>
+          <t>7th Annual RCF-ECGI Corporate Finance and Governance Conference</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Federal Reserve Bank of Philadelphia, Philadelphia, PA</t>
+          <t>Madrid, Spain, and virtually</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>€350 in person, €50 online option</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Interlinkages of the fintech sector and the broader financial system, economic consequences and impacts, regulatory implications of the fintech sector</t>
+          <t>capital structure, corporate and securities law, corporate culture, corporate failure, corporate finance and public policy, corporate governance, corporate restructuring, corporate social responsibility, crowdfunding, dividends, payout policy, and repurchases, entrepreneurial finance, family business, financial contracting, financial intermediation, financial literacy, fintech, fraud, innovation, IPOs and SEOs, mergers and acquisitions, misconduct, private debt, private equity, trade credit, socially responsible investments, sustainable finance, real options, venture capital</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Aarhus Finance Forum 2026</t>
+          <t>Fintech and Financial Institutions Research Conference</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Aarhus, Denmark</t>
+          <t>Federal Reserve Bank of Philadelphia, Philadelphia, PA</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>375 DKK (approx. 50 Euros)</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Financial Decisions under Uncertainty and Ambiguity, Household Finance, Real Estate Finance, Corporate Finance, Climate Finance, Digital Finance, Asset Pricing</t>
+          <t>Economic consequences and impacts of the fintech sector, regulatory implications of the fintech sector</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>15th CDI Conference on Derivatives</t>
+          <t>Aarhus Finance Forum 2026</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Montreal, Canada</t>
+          <t>Aarhus, Denmark</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>375 DKK</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Financial Decisions under Uncertainty and Ambiguity, Household Finance, Real Estate Finance, Corporate Finance, Climate Finance, Digital Finance, Asset Pricing</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Conference on CSR, the Economy and Financial Markets</t>
+          <t>15th CDI Conference on Derivatives</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2026-11-05</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Düsseldorf, Germany</t>
+          <t>Montreal, Canada</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>€ 150 for regular participants; € 100 for PhD students</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Climate risk and pricing; Role of financial markets, banks, institutional investors in CSR; Effects of CSR on valuation, performance, cost of capital, funding and capital structure; Socio-economic aspects and their implications for companies and financial markets; Corporate governance and CSR; Risk management and CSR; CSR reporting and disclosure; ESG backlash and politicization; Sustainability strategy under new constraints; Measurement: information content and reliability of ESG indices; CSR activities and the economy</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026 Vietnam Symposium on Global Economy (VSGE2026)</t>
+          <t>Conference on CSR, the Economy and Financial Markets</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City, Vietnam</t>
+          <t>Düsseldorf, Germany</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>€150 for regular participants, €100 for PhD students</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Geopolitical, macroeconomic policy, and development; trade, foreign direct investment, and global value chain; climate change, green transition, and public finance; finance, stability, and sustainable investment; digitalization, labor markets, and social protection; urbanization, regional development and resilience; AI, growth, economic impacts, and government policies; global governance, institutions, and international cooperation.</t>
+          <t>Climate risk and pricing, Role of financial markets, banks, institutional investors in CSR, Effects of CSR on valuation, performance, cost of capital, funding and capital structure, Socio-economic aspects and their implications for companies and financial markets, Corporate governance and CSR, Risk management and CSR, CSR reporting and disclosure, ESG backlash and politicization, Sustainability strategy under new constraints, Measurement: information content and reliability of ESG indices, CSR activities and the economy</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>21st Annual Conference on Asia-Pacific Financial Markets (CAFM)</t>
+          <t>2026 Vietnam Symposium on Global Economy (VSGE2026)</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2026-12-10</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>CONRAD Seoul</t>
+          <t>Ho Chi Minh City, Vietnam</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3335,34 +3311,34 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>All areas of finance</t>
+          <t>Geopolitical, macroeconomic policy, and development; Trade, foreign direct investment, and global value chain; Climate change, green transition, and public finance; Finance, stability, and sustainable investment; Digitalization, labor markets, and social protection; Urbanization, regional development and resilience; AI, growth, economic impacts, and government policies; Global governance, institutions, and international cooperation.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>India Finance Conference (IFC) 2026</t>
+          <t>21st Annual Conference on Asia-Pacific Financial Markets (CAFM)</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2026-12-21</t>
+          <t>2026-12-10</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>2026-12-23</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Indian Institute of Management Bangalore</t>
+          <t>CONRAD Seoul</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3372,34 +3348,34 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Theoretical and empirical asset pricing, Corporate finance, capital structure and dividend policy, Asset allocation and investment management, Financial crises, systemic risk and macro-finance, Quality of financial reporting and adoption of IFRS, Corporate governance, executive compensation and ownership structure, Computational finance and financial econometrics, Financial Econometrics, Financial risk analytics and management, Market microstructure and algorithmic trading, Financial policy choice, institutions and regulation, Financial Analytics, ESG, Climate Finance, Blended Finance, Insurance / Reinsurance / Pension Funds, Enhancing liquidity in commodity derivatives markets, Financial Literacy and Financial Education</t>
+          <t>All areas of finance</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Edinburgh Financial Technology Conference</t>
+          <t>India Finance Conference (IFC) 2026</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-12-21</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-12-23</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Edinburgh</t>
+          <t>Indian Institute of Management Bangalore</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3409,34 +3385,34 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>The application of AI and Machine Learning in finance, The application of distributed ledger technologies in finance, Cryptofinance, Cyber risk in finance, The microstructure of modern financial markets (algorithmic/high frequency trading, dark trading, blockchain settlements etc.), Behavioural economics in financial technology, Alternative data (structured and unstructured datasets), Crowdsourcing and investment strategy, New exchange traded financial derivatives, Financial stability risks from the development of FinTech, RegTech, Open banking</t>
+          <t>Theoretical and empirical asset pricing, Corporate finance, capital structure and dividend policy, Asset allocation and investment management, Financial crises, systemic risk and macro-finance, Quality of financial reporting and adoption of IFRS, Corporate governance, executive compensation and ownership structure, Computational finance and financial econometrics, Financial Econometrics, Financial risk analytics and management, Market microstructure and algorithmic trading, Financial policy choice, institutions and regulation, Financial Analytics, ESG, Climate Finance, Blended Finance, Insurance / Reinsurance / Pension Funds, Enhancing liquidity in commodity derivatives markets, Financial Literacy and Financial Education</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>5th Conference in Sustainable Finance</t>
+          <t>Edinburgh Financial Technology Conference</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>University of Luxembourg</t>
+          <t>Edinburgh</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -3446,34 +3422,34 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Any topic in sustainable finance</t>
+          <t>The application of AI and Machine Learning in finance, The application of distributed ledger technologies in finance, Cryptofinance, Cyber risk in finance, The microstructure of modern financial markets: algorithmic/high frequency trading, dark trading, blockchain settlements etc., Behavioural economics in financial technology, Alternative data (structured and unstructured datasets), Crowdsourcing and investment strategy, New exchange traded financial derivatives, Financial stability risks from the development of FinTech, RegTech, Open banking</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>7th CEAR-RSI Household Finance Workshop</t>
+          <t>5th Conference in Sustainable Finance</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2026-11-13</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>2026-11-14</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>HEC Montréal</t>
+          <t>University of Luxembourg</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3483,34 +3459,34 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Consumption-saving decisions and investment choices, Financial literacy and education, Pensions and retirement, Financial planning and advice, Financial delinquency and bankruptcy, Household insurance and risk management</t>
+          <t>Any topic in sustainable finance</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Next-Gen AI and Autonomous Finance (NGAI) workshop</t>
+          <t>7th CEAR-RSI Household Finance Workshop</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-11-14</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Rennes School of Business, Rennes, France</t>
+          <t>HEC Montréal</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3520,34 +3496,34 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Autonomous agents &amp; decision-making in finance, AI-driven trading, portfolio optimization &amp; market microstructure, Risk, robustness, and model governance (validation, monitoring, compliance), Ethics, fairness, transparency &amp; societal impacts of financial AI, Financial decision making and AI, Bias and stereotyping in relation to AI driven finance, AI, money and financial value formation</t>
+          <t>Consumption-saving decisions and investment choices, Financial literacy and education, Pensions and retirement, Financial planning and advice, Financial delinquency and bankruptcy, Household insurance and risk management</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>12th Annual ICGS Conference</t>
+          <t>Next-Gen AI and Autonomous Finance (NGAI) workshop</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>HEC Montréal (Quebec, Canada)</t>
+          <t>Rennes School of Business, Rennes, France</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3557,108 +3533,108 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Behavioral perspectives on executives, boards, investors, and other governance actors; Institutional and political approaches in governance; Implications of AI adoption for governance; Evolving forms of activism/engagement from investors and stakeholders; Reconfiguration of governance systems under geopolitical crises; Governance mechanisms for managing state-firm relations.</t>
+          <t>Autonomous agents &amp; decision-making in finance; AI-driven trading, portfolio optimization &amp; market microstructure; Risk, robustness, and model governance; Ethics, fairness, transparency &amp; societal impacts of financial AI; Financial decision making and AI; Bias and stereotyping in relation to AI driven finance; AI, money and financial value formation.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Vienna Festival of Finance Theory 2026</t>
+          <t>12th Annual ICGS Conference</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Vienna, Austria</t>
+          <t>HEC Montréal (Quebec, Canada)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>65 EUR</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Corporate finance theory, financial intermediation theory</t>
+          <t>Behavioral perspectives on governance, Institutional and political approaches to governance, Implications of AI adoption for governance, Evolving forms of activism/engagement, Reconfiguration of governance systems under geopolitical crises, Governance mechanisms for managing state-firm relations</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Cross Country Perspectives in Finance (CCPF) Conference</t>
+          <t>Vienna Festival of Finance Theory 2026</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>both online and on-site (Nanjing, China)</t>
+          <t>Vienna, Austria</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>65 EUR</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>credit, banking, asset pricing, market liquidity, corporate finance, corporate governance, entrepreneurial finance</t>
+          <t>Corporate finance theory, financial intermediation theory</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Private Capital Symposium 2026</t>
+          <t>11th (2026) Cross Country Perspectives in Finance (CCPF) Conference</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>London Business School, London</t>
+          <t>both online and on-site (Nanjing, China)</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -3668,7 +3644,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Research on private equity, venture capital, and broader private market themes</t>
+          <t>credit, banking, asset pricing, market liquidity, corporate finance, corporate governance, entrepreneurial finance in an international context</t>
         </is>
       </c>
     </row>
@@ -3742,7 +3718,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Asset pricing, macro-finance, impact of institutional features on capital market dynamics</t>
+          <t>asset pricing, macro-finance, impact of institutional features on capital market dynamics</t>
         </is>
       </c>
     </row>
@@ -3816,7 +3792,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Investor behavior, behavior of different investor types, market microstructure and investor trading behavior, behavioral biases and performance of investment strategies, household consumption, borrowing, saving, and portfolio choice, investor education, financial literacy and sophistication, behavior of finance professionals and impact of professional advice, biological, psychological, and cultural foundations of investor behavior, influence of analysts, media, and news coverage on investment decisions, social influence and networks in finance, impact of investor behavior on corporate policies and decision-making</t>
+          <t>Investor behavior, Behavior of different investor types, Market microstructure and investor trading behavior, Behavioral biases and performance of investment strategies, Household consumption, borrowing, saving, and portfolio choice, Investor education, financial literacy, and sophistication, Behavior of finance professionals and the impact of professional advice, Biological, psychological, and cultural foundations of investor behavior, The influence of analysts, media, and news coverage on investment decisions, Social influence and networks in finance, Impact of investor behavior on corporate policies and decision-making</t>
         </is>
       </c>
     </row>
@@ -3885,7 +3861,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>$75</t>
+          <t>$75 USD</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -3897,7 +3873,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>11th SDU Finance Workshop on Corporate Finance</t>
+          <t>11th SDU Finance Workshop on Corporate Finance -- Dynamics, Uncertainty, and Strategic Decisions</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -3964,7 +3940,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>topics from all areas of finance including asset pricing, corporate finance, financial intermediation, investments, Canadian financial markets, insurance, household finance, sustainable finance, fintech, and AI</t>
+          <t>Topics from all areas of finance including asset pricing, corporate finance, financial intermediation, investments, Canadian financial markets, insurance, household finance, sustainable finance, fintech and AI</t>
         </is>
       </c>
     </row>
@@ -3996,19 +3972,19 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>£50</t>
+          <t>£50 GBP</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>All areas of finance</t>
+          <t>Papers from all areas of finance</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Sustainability, Technology, and the Transformation of Accounting and Finance (STTAF26)</t>
+          <t>International Conference on Sustainability, Technology, and the Transformation of Accounting and Finance (STTAF 2026)</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -4075,7 +4051,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Accounting, Finance, Banking (theoretical and empirical studies)</t>
+          <t>All areas of Accounting, Finance, and Banking, encompassing both theoretical and empirical studies</t>
         </is>
       </c>
     </row>
@@ -4112,7 +4088,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>forecasting financial variables with AI, asset allocation and asset management with AI, AI-based factor models, natural language processing and large language models in finance, and AI applications in corporate finance</t>
+          <t>forecasting financial variables with AI, asset allocation and asset management with AI, AI-based factor models, natural language processing and large language models in finance, AI applications in corporate finance</t>
         </is>
       </c>
     </row>
@@ -4304,39 +4280,15 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>12th IWH-FIN-FIRE Workshop on “Challenges to Financial Stability”</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>2026-05-11</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
-        <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>2026-08-25</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>Halle/Saale, Germany</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>regulation and financial intermediation, corporate finance, law, politics and finance, monetary policy, inflation and financial resilience, macroprudential policy and real estate, financial networks and systemic risk, pricing of climate risk in financial markets, ecological hazards and the behaviour of firms and households, governance of financial firms and markets, private credit and risk transfer</t>
-        </is>
-      </c>
+          <t>I apologize, but it seems that you haven't provided the text of the announcement. Please share the text, and I'll be happy to extract the required information for you.</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr"/>
+      <c r="C106" t="inlineStr"/>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -4366,7 +4318,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>$50</t>
+          <t>$50 USD</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -4378,39 +4330,15 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>11th Bank of Finland and European Systemic Risk Board Joint Conference on AI and Systemic Risk Analytics</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>2026-03-31</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>2026-06-03</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>Bank of Finland, Helsinki</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t>Use of Large Language Models (LLM) and trustworthy AI, AI and changing interdependencies in the financial markets, Cyber security and operational risks as sources of systemic risk, AI and Quantum Computing as potential source of new systemic risks, Use of AI with big data for systemic risk analytics, Risks and opportunities stemming from disruptive innovations in financial technology (FinTech), Analysing emerging risks from interconnectedness of the financial system, Identifying risks from market-based finance, Modelling geopolitical risks, Using systemic risk analytics to support macro-prudential policy and regulation, Evidence of macroprudential policy measures</t>
-        </is>
-      </c>
+          <t>It appears that the text of the announcement was not included in your message. Please provide the text of the call for papers so I can extract the required information for you.</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr"/>
+      <c r="C108" t="inlineStr"/>
+      <c r="D108" t="inlineStr"/>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -4556,7 +4484,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Finance and Economics</t>
+          <t>Finance, Economics</t>
         </is>
       </c>
     </row>
@@ -4593,7 +4521,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Monetary Policy Transmission, Expectations, and Communication; Inflation and Price Dynamics; Macro-Finance and Financial Stability; Fiscal–Monetary Interactions and Policy Making; International Macroeconomics, Trade, and Geoeconomics; Firms, Productivity, and the Real Economy; Data, Methods, and Artificial Intelligence</t>
+          <t>Monetary Policy Transmission, Expectations, and Communication, Inflation and Price Dynamics, Macro-Finance and Financial Stability, Fiscal–Monetary Interactions and Policy Making, International Macroeconomics, Trade, and Geoeconomics, Firms, Productivity, and the Real Economy, Data, Methods, and Artificial Intelligence</t>
         </is>
       </c>
     </row>
@@ -4667,7 +4595,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Interaction between financial and labor markets, technological innovation, job-skill matches, firms’ employment policies, role of employees in governance and financing of companies, responses of wages and employment to shocks, risk-sharing arrangements between firms and workers</t>
+          <t>Interaction between financial and labor markets, technological innovation, job-skill matches, firms’ employment policies, role of employees in governance and financing of companies, responses of wages, employment, and career trajectories to shocks, risk-sharing arrangements between firms and workers</t>
         </is>
       </c>
     </row>
@@ -4741,7 +4669,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Fintech and Financial Institutions, Regulatory framework revisions, CBDC blockchains, and stablecoins, Sovereign bonds and sovereign bond capital regulation, Payment systems and European sovereignty, Safe assets and exchange rate dynamics under world polarization, Private credit and financial stability, Climate regulation U-turn and implications for climate finance, Defence policy needs and European financial architecture</t>
+          <t>Fintech and Financial Institutions, Regulatory framework revisions, CBDC blockchains and stablecoins, Sovereign bonds and sovereign bond capital regulation, Payment systems and European sovereignty, Safe assets and exchange rate dynamics under world polarization, Private credit and financial stability, Climate regulation U-turn and implications for climate finance, Defence policy needs and European financial architecture</t>
         </is>
       </c>
     </row>
@@ -4810,7 +4738,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>£65</t>
+          <t>£65 GBP</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -4842,17 +4770,17 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Seattle, Washington | UW Foster School of Business</t>
+          <t>Seattle, Washington</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>USD $80 per paper</t>
+          <t>80 USD</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>All areas of finance, particularly submissions from junior faculty and preliminary papers</t>
+          <t>All areas of finance</t>
         </is>
       </c>
     </row>
@@ -4963,7 +4891,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>sustainable finance, corporate governance, sustainability</t>
+          <t>Sustainable finance and the intersection of corporate governance and sustainability</t>
         </is>
       </c>
     </row>
@@ -5000,7 +4928,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Energy, Sustainability, Fintech including AI, Climate change, Alternative Investments, Asset &amp; Wealth Management, Asset Allocation, Sovereign Funds, Hedge Funds, ETFs, SWFs, Banking &amp; Financial Services, Corporate Governance, Executive Compensation, Country Risk, Debt Issues, Insurance, Reinsurance, Derivatives, Financial Engineering, E-Business, E-Finance, Social Media, Emerging Markets, Entrepreneurship, Venture Capital, Ethics, Legal, Regulatory Issues, Financial Crises, Financial Technology, Foreign Currency Issues, Future of Global Economy, Global Trade Issues, IPOs, SEOs, Stock Buybacks, Mergers and Acquisitions, Non-Traditional Banking, Portfolio Flows, Private Equity, Real Estate, Valuation, Portfolio Management, and Managing Financial Risk.</t>
+          <t>Energy, Sustainability, Fintech including AI, Climate change, Alternative Investments, Asset &amp; Wealth Management, Asset Allocation/Sovereign Funds/Hedge Funds/ETFs/SWFs, Banking &amp; Financial Services, Corporate Governance/Executive Compensation, Country Risk/Debt Issues/Insurance/Reinsurance, Derivatives/Financial Engineering, E-Business/E-Finance/Social Media, Emerging Markets/BRICS, Entrepreneurship/Venture Capital Global Perspectives, Ethics/Legal/Regulatory, Financial Crises and Bubbles, Financial Technology including AI, Foreign Currency Issues, Future of Global Economy, Global Trade Issues, IPOs/SEOs/Stock buybacks/Privatization, Market Behavior Efficiency/Inefficiency, Mergers and Acquisitions, Non-Traditional Banking &amp; Financial Services, Portfolio Flows and Foreign Direct Investment, Private Equity, Real estate - global perspectives, Valuation, Portfolio Management and Managing Financial Risk</t>
         </is>
       </c>
     </row>
@@ -5037,7 +4965,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Asset management, Asset pricing, Papers that bridge asset management and asset pricing</t>
+          <t>Asset management, asset pricing, papers bridging both areas</t>
         </is>
       </c>
     </row>
@@ -5069,12 +4997,12 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>70 USD</t>
+          <t>USD 70</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Asset pricing, financial intermediation, investments, Demand Based Asset Pricing, Inelastic Markets Hypothesis, New Methods in Asset Pricing (Machine Learning, AI, unstructured data), Time series and Cross-Sectional Predictability, Portfolio Allocation for Long Term Investors, Retirement decisions and choices, Behavioral finance</t>
+          <t>Demand Based Asset Pricing, Inelastic Markets Hypothesis, New Methods in Asset Pricing (Machine Learning, Artificial Intelligence (AI), unstructured data), Time series and Cross-Sectional Predictability, Portfolio Allocation for Long Term Investors, Retirement decisions and choices, Behavioral finance</t>
         </is>
       </c>
     </row>
@@ -5111,7 +5039,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>AI, asset pricing, banking, behavioral finance, big data, blockchain, CBDCs, compliance, crowdfunding, cryptocurrencies, cybersecurity, decentralized finance, digital finance, embedded finance, fintech, financial infrastructure, financial inclusion, financial innovation, financial intermediation, financial markets, household finance, insurtech, machine learning, market microstructure, payments, platforms, regulation, risk management, stablecoins, tokenization, text analytics</t>
+          <t>AI, asset pricing, banking, behavioral finance, big data, blockchain, CBDCs, compliance, crowdfunding, cryptocurrencies, cybersecurity, decentralized finance, digital finance, embedded finance, fintech, financial infrastructure, financial inclusion, financial innovation, financial intermediation, financial markets, household finance, insurtech, machine learning, market microstructure, payments, platforms, regulation, risk management, stablecoins, tokenization, text analytics.</t>
         </is>
       </c>
     </row>
@@ -5143,12 +5071,12 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>$50 USD (FMA-members) / $60 USD (non-members)</t>
+          <t>$50 USD (FMA-members), $60 USD (non-members)</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>High-quality papers in the fields of finance and accounting that inform practice, advance academic research, address contemporary global issues, and introduce new hypotheses.</t>
+          <t>Inform practice and advance the frontiers of academic research in directions relevant to practice; Address issues that are relevant to contemporary issues globally and for policy formation and assessment; Introduce new hypotheses that have the potential to stimulate additional research</t>
         </is>
       </c>
     </row>
@@ -5180,12 +5108,12 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0 GBP</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Sustainable finance, interdisciplinary research</t>
+          <t>Unpublished research papers on any topic related to sustainable finance, interdisciplinary research that draws together approaches and perspectives from different disciplines</t>
         </is>
       </c>
     </row>
@@ -5222,7 +5150,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Cryptofinance, cryptocurrencies, digital finance, blockchain economics, AI for finance, corporate finance, alternative investments</t>
+          <t>Cryptofinance, blockchain economics, digital finance, FinTech, corporate finance, entrepreneurship, alternative investments</t>
         </is>
       </c>
     </row>
@@ -5259,7 +5187,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Non-academic-friendly summaries of research, pressing questions informed by academic research, sustainability issues</t>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -5333,7 +5261,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>sustainable finance, green finance, climate finance, international finance</t>
+          <t>Sustainable finance, green finance, climate finance, international finance</t>
         </is>
       </c>
     </row>
@@ -5377,7 +5305,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>22nd Annual Conference of the Asia-Pacific Association of Derivatives</t>
+          <t>The 22nd Annual Conference of the Asia-Pacific Association of Derivatives</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -5444,7 +5372,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>The impact of investment in AI and supporting technologies on corporate earnings and share prices; the effects of AI on portfolio choices and trading behavior; the role of AI in creating new measures of economic activity; the uses of AI in financial market regulation; the consequences of AI for the financial advice industry; the macroeconomic effects of AI on economy-wide discount rates</t>
+          <t>The impact of investment in AI and supporting technologies on corporate earnings and share prices; effects of AI on portfolio choices and trading behavior of financial market participants; role of AI in creating new measures of economic activity; uses of AI in financial market regulation; consequences of AI for the financial advice industry; macroeconomic effects of AI on economy-wide discount rates</t>
         </is>
       </c>
     </row>
@@ -5513,12 +5441,12 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>450 euros</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>Venture capital; private equity and buyouts; Business angels and early-stage financing; Crowdfunding; token offerings and digital finance; Entrepreneurial banking and credit relationships; Corporate governance, contracts, and monitoring; Financial innovation; FinTech and AI in entrepreneurial finance; ESG, sustainability, and impact finance; Entrepreneurial ecosystems and regional financing gaps; Entrepreneurial risk-taking and behavioral finance; Impact assessment for publicly supported financial instruments and their real effects and societal outcomes.</t>
+          <t>Venture capital; private equity, and buyouts; Business angels and early-stage financing; Crowdfunding; token offerings, and digital finance; Entrepreneurial banking and credit relationships; Corporate governance, contracts, and monitoring; Financial innovation; FinTech, and AI in entrepreneurial finance; ESG, sustainability, and impact finance; Entrepreneurial ecosystems and regional financing gaps; Entrepreneurial risk-taking and behavioral finance; Impact assessment for publicly supported financial instruments</t>
         </is>
       </c>
     </row>
@@ -5550,12 +5478,12 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>0 USD</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>Maturity and liquidity transformation by banks, broker-dealers, money market mutual funds, and other financial intermediaries; Repo markets and their clearing institutions; Theories of frictions and fragility in short-term funding markets; Effects of regulation and central bank intervention on funding markets; Securities lending; Money creation and the demand for safe assets; Fintech and encrypted currency</t>
+          <t>Maturity and liquidity transformation, Repo markets and their clearing institutions, Theories of frictions and fragility in short-term funding markets, Effects of regulation and central bank intervention on funding markets, Securities lending, Money creation and the demand for safe assets, Fintech and encrypted currency</t>
         </is>
       </c>
     </row>
@@ -5629,7 +5557,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Buyouts, distressed securities, mezzanine financing, special situations, private credit, venture capital, real estate, real assets</t>
+          <t>Private equity, buyouts, distressed securities, mezzanine financing, special situations, private credit, venture capital, real estate, real assets</t>
         </is>
       </c>
     </row>
@@ -5666,7 +5594,7 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Corporate Finance, including mergers and acquisitions, corporate governance, and financial institutions</t>
+          <t>Corporate Finance</t>
         </is>
       </c>
     </row>
@@ -5735,12 +5663,12 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>$50 USD</t>
+          <t>50 USD</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>Papers on any area of finance, panel discussions, special sessions, tutorials</t>
+          <t>Papers on any area of finance, proposals for panel discussions, special sessions, or tutorials</t>
         </is>
       </c>
     </row>
@@ -5777,7 +5705,7 @@
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>Original empirical and theoretical papers in accounting and finance, including banking, with a focus on significant and impactful issues within these fields</t>
+          <t>Original empirical and theoretical papers in accounting and finance, with a focus on significant and impactful issues within these fields</t>
         </is>
       </c>
     </row>
@@ -5814,7 +5742,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Risk Governance in the boardroom, Risk Governance and the monitoring role of supervisory boards, Balancing risk and opportunity, Stakeholder influence on decision-making, Sustainability and Risk Governance, Understanding black swans in decision-making, Strategic resilience, Risk strategies on bank boards, Tackling digitalization-related risks, Role of artificial intelligence in decisions, Machine learning in decision-making</t>
+          <t>Risk Governance in the boardroom, Risk Governance and the monitoring role of supervisory boards, Balancing risk and opportunity, Stakeholder influence on board decision-making, Sustainability and Risk Governance, Understanding black swans, Strategic resilience, Considering risk strategies on bank boards, Tackling digitalization-related risks, The role of artificial intelligence for board decisions</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5786,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>9th Annual J.P. Morgan Center International Commodities Symposium</t>
+          <t>CU Denver 9th Annual J.P. Morgan Center International Commodities Symposium</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -5888,7 +5816,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>Commodity business, energy, metals and minerals, agriculture, commodity futures, derivatives</t>
+          <t>Broad global commodity sectors (energy, metals and minerals, and agriculture), commodity futures, derivatives, and related research topics</t>
         </is>
       </c>
     </row>
@@ -6031,7 +5959,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>$75 USD (FMA-members) and $85 USD (non-members)</t>
+          <t>$75 USD (FMA-members), $85 USD (non-members)</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -6142,7 +6070,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>£50 GBP</t>
+          <t>£50</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -6221,7 +6149,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Entrepreneurship and innovation, Scaling frontier technologies, Industrial policy and innovation, University-industry collaboration, Global innovation networks, Innovation finance, Universities, governments, and policy in the new geopolitical era</t>
+          <t>Entrepreneurship and innovation, scaling frontier technologies, industrial policy and innovation, university-industry collaboration, global innovation networks, innovation finance, universities, governments, and policy in the new geopolitical era</t>
         </is>
       </c>
     </row>
@@ -6258,7 +6186,7 @@
       </c>
       <c r="G158" t="inlineStr">
         <is>
-          <t>(1) Empirical finance with AI and Big Data applications (e.g., alternative data) (2) New empirical method development in machine learning and financial econometrics (3) Blockchain technology, digital assets, and frontier FinTech topics</t>
+          <t>Empirical finance with AI and Big Data applications, New empirical method development in machine learning and financial econometrics, Blockchain technology, digital assets, and frontier FinTech topics</t>
         </is>
       </c>
     </row>
@@ -6295,7 +6223,7 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>New Technologies and Their Implications for Monetary Policy and Financial Stability, AI and automation impact on inflation dynamics, risks to financial stability from technological developments, adaptation of central banks' toolkits, transformation of financial markets, macroprudential supervision, monetary policy transmission mechanism, optimization of monetary policy decision-making using AI</t>
+          <t>New Technologies and Their Implications for Monetary Policy and Financial Stability, AI and automation impact on inflation dynamics, financial stability risks from technological developments, central banks' toolkits in an AI-driven economy, transformation of financial markets, macroprudential supervision risks and opportunities, effects of technological advances on monetary policy transmission mechanism, use of AI in optimizing monetary policy decision making</t>
         </is>
       </c>
     </row>
@@ -6332,7 +6260,7 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>All aspects of behavioral finance, including financial behavior of individuals, groups, and organizations, market dynamics, and intersection of these areas</t>
+          <t>all aspects of behavioral finance, financial behavior of individuals, financial behavior of groups and organizations, dynamics of markets</t>
         </is>
       </c>
     </row>
@@ -6438,7 +6366,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>75 USD</t>
+          <t>$75 USD</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -6480,7 +6408,7 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>Uses of AI by firms in corporate finance, AI use in trading and asset management, AI use by banks and other credit providers, AI use in financial forecasting, AI use for understanding consumer financial behavior, AI and labor replacement vs. augmentation, Financial market and macroeconomic implications of AI use, AI, financial stability, and disparities, Frictions and market failures in AI adoption/use and regulatory solutions</t>
+          <t>Opportunities and risks of AI technologies in Finance, uses of AI by firms in corporate finance, AI use in trading and asset management, AI use by banks and credit providers, AI in financial forecasting, AI and consumer financial behavior, AI and labor replacement vs. augmentation, financial market implications of AI, risks to financial stability, frictions in AI adoption</t>
         </is>
       </c>
     </row>
@@ -6507,17 +6435,17 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>Coogee Beach (Sydney, Australia)</t>
+          <t>Coogee Beach, Sydney, Australia</t>
         </is>
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>0 USD</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>All areas of Finance with a special focus on Corporate Finance, including banking, household and entrepreneurial finance</t>
+          <t>All areas of Finance, with a special focus on Corporate Finance, including banking, household and entrepreneurial finance</t>
         </is>
       </c>
     </row>
@@ -6554,46 +6482,22 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>Theoretical and empirical papers in banking and financial intermediation</t>
+          <t>theoretical and empirical papers in banking and financial intermediation</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>CCA-ESCP Workshop on Financial Institutions and Corporate Finance</t>
-        </is>
-      </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>2026-02-14</t>
-        </is>
-      </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>2026-06-04</t>
-        </is>
-      </c>
-      <c r="D167" t="inlineStr">
-        <is>
-          <t>2026-06-05</t>
-        </is>
-      </c>
-      <c r="E167" t="inlineStr">
-        <is>
-          <t>ESCP Business School - Turin Campus</t>
-        </is>
-      </c>
-      <c r="F167" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G167" t="inlineStr">
-        <is>
-          <t>Interactions among banks, non-bank intermediaries, and capital markets; Effects of technological innovation; Consequences of bank regulatory and supervisory reforms; Determinants of financial fragility, liquidity transformation, and systemic risk; Climate, sustainability, and transition finance; Corporate investment, capital structure, and liquidity management; Governance, ownership structures, incentives, and diversity; Monetary-policy transmission through banks and non-banks; Household and entrepreneurial finance; Impacts of geopolitical, political-economy, and policy shocks in finance</t>
-        </is>
-      </c>
+          <t>Please provide the text of the announcement so I can extract the required information for you.</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr"/>
+      <c r="C167" t="inlineStr"/>
+      <c r="D167" t="inlineStr"/>
+      <c r="E167" t="inlineStr"/>
+      <c r="F167" t="inlineStr"/>
+      <c r="G167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -6746,7 +6650,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>10th Vietnam International Conference in Finance</t>
+          <t>The 10th Vietnam International Conference in Finance</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -6813,7 +6717,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>all areas of finance, financial economics</t>
+          <t>Innovative research across all areas of finance</t>
         </is>
       </c>
     </row>
@@ -6850,7 +6754,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>NLP &amp; large language models; Speech and multimedia analysis; AI agents &amp; automation; Machine learning &amp; predictive analytics; Big data &amp; computational methods; The role of AI in corporate decision-making and other aspects of financial and labor markets; Ethics, policy, and regulation</t>
+          <t>NLP &amp; large language models, Speech and multimedia analysis, AI agents &amp; automation, Machine learning &amp; predictive analytics, Big data &amp; computational methods, The role of AI in corporate decision-making and other aspects of financial and labor markets, Ethics, policy, and regulation</t>
         </is>
       </c>
     </row>
@@ -6887,7 +6791,7 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>Banks’ ESG and Climate Responsibilities; Banks as ESG and Climate Gatekeepers for Corporations; Banks, Climate Risk, and Financial Stability; Regulations, ESG, and Climate Risk; Central Banks, Banking Regulations, and Green Finance</t>
+          <t>Banks’ ESG and Climate Responsibilities, Banks as ESG and Climate Gatekeepers for Corporations, Banks, Climate Risk, and Financial Stability, Regulations, ESG, and Climate Risk, Central Banks, Banking Regulations, and Green Finance</t>
         </is>
       </c>
     </row>
@@ -6998,7 +6902,7 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>Energy and commodity finance, financial and operational risk analysis, decision making, optimization for sustainable ecosystems</t>
+          <t>Economics, finance, mathematics, operations, risk management, energy and commodity sourcing, processing, trading, financial and operational risk analysis, decision making, optimization for sustainable ecosystems</t>
         </is>
       </c>
     </row>
@@ -7036,80 +6940,6 @@
       <c r="G179" t="inlineStr">
         <is>
           <t>Big Data &amp; Information Efficiency, AI, Automation &amp; Liquidity, Modern Market Design, Blockchain &amp; Digital Market Microstructure, Stability, Systemic Risk &amp; Real Effects, Policy, Regulation &amp; SupTech</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D180" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E180" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F180" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G180" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D181" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E181" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F181" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G181" t="inlineStr">
-        <is>
-          <t>N/A</t>
         </is>
       </c>
     </row>

</xml_diff>